<commit_message>
Implement client signup, hybrid password login, status toggles, and remove OTP
</commit_message>
<xml_diff>
--- a/data/work_records.xlsx
+++ b/data/work_records.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -522,99 +522,6 @@
       <c r="K2" t="inlineStr">
         <is>
           <t>Completed</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>W002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>C001</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Umashankar Pradhan</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>S003</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>YouTube Shorts</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" t="n">
-        <v>800</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1600</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>W003</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>C001</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Umashankar Pradhan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>S010</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>YouTube Video Edit</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" t="n">
-        <v>800</v>
-      </c>
-      <c r="I4" t="n">
-        <v>1600</v>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Pending</t>
         </is>
       </c>
     </row>

</xml_diff>